<commit_message>
docs: update F04 test execution results and add 30 F05 30 F06 test case - 23130082 - NguyenTruongGiang
</commit_message>
<xml_diff>
--- a/planning/Test_Plan_DiDongViet.xlsx
+++ b/planning/Test_Plan_DiDongViet.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HUONG DAN" sheetId="1" r:id="Rdfd09bc93b524c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHAN CONG" sheetId="2" r:id="Rca956506e69d45cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST DESIGN" sheetId="3" r:id="R0ee187659bf34e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV1 - TEST CASE" sheetId="4" r:id="R9ee0f4224c304090"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV2 - TEST CASE" sheetId="5" r:id="R58244075e7a7445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV3 - TEST CASE" sheetId="6" r:id="R299e1b15b1af4539"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV4 - TEST CASE" sheetId="7" r:id="Rb142196f01964ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV5 - TEST CASE" sheetId="8" r:id="Re2e6528171954472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TONG QUAN" sheetId="9" r:id="R7ad9ddab4510470d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUTOMATION PLAN" sheetId="10" r:id="Re9bc8133a83949f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NGUON &amp; LUU Y" sheetId="11" r:id="R70ba88ecb7204ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HUONG DAN" sheetId="1" r:id="R889afb8aadc84f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHAN CONG" sheetId="2" r:id="R0431e473c8ac4118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST DESIGN" sheetId="3" r:id="R3a37aa212c72425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV1 - TEST CASE" sheetId="4" r:id="R1b12234cadcd462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV2 - TEST CASE" sheetId="5" r:id="Rc3899d4f2a504db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV3 - TEST CASE" sheetId="6" r:id="Rd353099f8885429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV4 - TEST CASE" sheetId="7" r:id="Rc78630370471431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV5 - TEST CASE" sheetId="8" r:id="R0f4038f2f665475c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TONG QUAN" sheetId="9" r:id="R3e99abdb7e754e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUTOMATION PLAN" sheetId="10" r:id="R5e17e8ccdf0843aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NGUON &amp; LUU Y" sheetId="11" r:id="R543ad1e6b8974653"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -158,7 +158,7 @@
         <x:color rgb="FF11613B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE1F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -168,7 +168,7 @@
         <x:color rgb="FF9A2121"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -178,7 +178,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -188,7 +188,7 @@
         <x:color rgb="FF11613B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE1F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -198,7 +198,7 @@
         <x:color rgb="FF9A2121"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -208,7 +208,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -218,7 +218,7 @@
         <x:color rgb="FF11613B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE1F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -228,7 +228,7 @@
         <x:color rgb="FF9A2121"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -238,7 +238,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -248,7 +248,7 @@
         <x:color rgb="FF11613B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE1F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -258,7 +258,7 @@
         <x:color rgb="FF9A2121"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -268,7 +268,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -278,7 +278,7 @@
         <x:color rgb="FF11613B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE1F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -288,7 +288,7 @@
         <x:color rgb="FF9A2121"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -298,7 +298,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -769,7 +769,7 @@
     </x:row>
     <x:row r="2" ht="31" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>Katalon Recorder làm bước khởi đầu • Chạy thử trong môi trường cho phép • Tuyệt đối không tạo giao dịch/lead thật</x:v>
+        <x:v>Automation Playwright trên giao diện thật • TV2 F04 (biến thể), F05 (giỏ), F06 (MUA NGAY) • Không tạo đơn/thanh toán thật</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
         <x:v>Katalon Recorder làm bước khởi đầu • Chạy thử trong môi trường cho phép • Tuyệt đối không tạo giao dịch/lead thật</x:v>
@@ -971,7 +971,7 @@
         <x:v>Thiết lập trình duyệt và công cụ</x:v>
       </x:c>
       <x:c r="D11" s="26" t="str">
-        <x:v>Chốt Katalon Recorder / Selenium + phiên bản; mở website không lỗi.</x:v>
+        <x:v>Chốt Playwright hoặc công cụ automation của nhóm, mở sản phẩm và thu thập selector ổn định.</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
         <x:v>Cả nhóm</x:v>
@@ -980,7 +980,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
-        <x:v>Chrome + Katalon Recorder</x:v>
+        <x:v>Chrome/Edge + Playwright</x:v>
       </x:c>
       <x:c r="H11" s="26" t="str">
         <x:v>Chưa làm</x:v>
@@ -998,7 +998,7 @@
         <x:v>Selector ổn định</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
-        <x:v>ID/CSS/xpath ổn định; kiểm tra assertion đúng đối tượng.</x:v>
+        <x:v>Locator riêng cho biểu tượng xe đẩy (F05) và nút MUA NGAY (F06); ưu tiên getByRole/text trên trang Samsung.</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
         <x:v>5 TV</x:v>
@@ -1007,7 +1007,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
-        <x:v>DevTools + Katalon</x:v>
+        <x:v>DevTools + Playwright</x:v>
       </x:c>
       <x:c r="H12" s="26" t="str">
         <x:v>Chưa làm</x:v>
@@ -1076,10 +1076,10 @@
         <x:v>Automation</x:v>
       </x:c>
       <x:c r="C15" s="26" t="str">
-        <x:v>TV2 biến thể/giỏ/mua kèm</x:v>
+        <x:v>TV2 biến thể / giỏ hàng / MUA NGAY</x:v>
       </x:c>
       <x:c r="D15" s="26" t="str">
-        <x:v>Assert SKU, số lượng và tổng tiền, không đi đến xác nhận thanh toán.</x:v>
+        <x:v>Assert SKU/màu, số lượng giỏ; riêng F06 MUA NGAY kiểm tra điều hướng, giá/tóm tắt sản phẩm, không đặt hàng.</x:v>
       </x:c>
       <x:c r="E15" s="26" t="str">
         <x:v>TV2</x:v>
@@ -1088,7 +1088,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G15" s="26" t="str">
-        <x:v>F04,F05,F06</x:v>
+        <x:v>Playwright; F04, F05, F06</x:v>
       </x:c>
       <x:c r="H15" s="26" t="str">
         <x:v>Chưa làm</x:v>
@@ -1468,7 +1468,7 @@
         <x:v>Nguồn trực tiếp</x:v>
       </x:c>
       <x:c r="F6" s="26" t="str">
-        <x:v>Đã giữ đúng 15 chức năng và phân công</x:v>
+        <x:v>15 chức năng phân công không trùng; F06 TV2 là MUA NGAY trước bước điền thông tin (không thuộc F07/F08/F14).</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="59" customHeight="1">
@@ -1609,6 +1609,26 @@
       </x:c>
       <x:c r="F13" s="26" t="str">
         <x:v>20–30 TC cho ít nhất một chức năng / TV; không có tối đa bắt buộc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Trang Samsung S25 Ultra 256GB</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>F05, F06</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Đã thấy nút MUA NGAY</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>F05 dùng biểu tượng giỏ; F06 dùng MUA NGAY trên cùng sản phẩm Samsung. Màn hình sau nhấn cần kiểm tra khi chạy; không tạo đơn.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1941,11 +1961,11 @@
       </x:c>
       <x:c r="I9" s="30" t="n">
         <x:f>COUNTIF('TV2 - TEST CASE'!M6:M35,"PASS")+COUNTIF('TV2 - TEST CASE'!M6:M35,"FAIL")+COUNTIF('TV2 - TEST CASE'!M6:M35,"BLOCKED")</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="J9" s="30" t="n">
         <x:f>COUNTIF('TV2 - TEST CASE'!M6:M35,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K9" s="30" t="str">
         <x:v>Cần xác minh</x:v>
@@ -2021,7 +2041,7 @@
         <x:v>Cấu hình và giỏ hàng</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
         <x:v>3</x:v>
@@ -2045,13 +2065,13 @@
         <x:v>Cần xác minh</x:v>
       </x:c>
       <x:c r="L11" s="30" t="str">
-        <x:v>Có điều kiện</x:v>
+        <x:v>Cao</x:v>
       </x:c>
       <x:c r="M11" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng.</x:v>
+        <x:v>Nút MUA NGAY đã thấy trên S25 Ultra; màn hình sau nhấn phải kiểm tra. Không đặt hàng thật.</x:v>
       </x:c>
       <x:c r="N11" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -2501,11 +2521,11 @@
       </x:c>
       <x:c r="I22" s="32" t="n">
         <x:f>SUM(I6:I20)</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="J22" s="32" t="n">
         <x:f>SUM(J6:J20)</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K22" s="32"/>
       <x:c r="L22" s="32"/>
@@ -2856,34 +2876,34 @@
         <x:v>TV2</x:v>
       </x:c>
       <x:c r="C11" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D11" s="26" t="str">
-        <x:v>Tính đúng điều kiện và giá combo</x:v>
+        <x:v>MUA NGAY từ trang sản phẩm, bảo toàn SKU, màu, giá trước bước điền khách hàng</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
-        <x:v>Thêm/bỏ món mua kèm; nhiều gói; số lượng; đổi biến thể chính</x:v>
+        <x:v>4 màu; 256/512GB/1TB có điều kiện; giá; trạng thái giỏ; Back/Forward; viewport; bấm lặp; không tạo đơn</x:v>
       </x:c>
       <x:c r="F11" s="26" t="str">
-        <x:v>Bảng quyết định; Pairwise</x:v>
+        <x:v>State Transition; Decision Table; Boundary Value; Equivalence Partitioning</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
-        <x:v>Sản phẩm có mục 'mua kèm'</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; chọn SKU khả dụng, không nhập dữ liệu thật</x:v>
       </x:c>
       <x:c r="H11" s="26" t="str">
-        <x:v>Sản phẩm chính và phụ kiện A/B</x:v>
+        <x:v>Samsung S25 Ultra 256GB và các màu; phiên bản 512GB/1TB nếu còn hàng; trạng thái giỏ</x:v>
       </x:c>
       <x:c r="I11" s="26" t="str">
-        <x:v>Tổng tiền, khuyến mãi và trạng thái đúng</x:v>
+        <x:v>Đi đến luồng mua đúng SKU, không tạo đơn/thanh toán chỉ từ thao tác MUA NGAY</x:v>
       </x:c>
       <x:c r="J11" s="26" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Cao</x:v>
       </x:c>
       <x:c r="K11" s="26" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="L11" s="26" t="str">
-        <x:v>Chưa xác minh</x:v>
+        <x:v>Đã thấy MUA NGAY; chưa xác minh màn hình sau nhấn</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="75" customHeight="1">
@@ -8431,7 +8451,7 @@
     </x:row>
     <x:row r="2" ht="31" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>Phụ trách: F04, F05, F06  •  Case đầu tiên của mỗi chức năng: 30  •  Chưa chạy, chưa xác minh UI</x:v>
+        <x:v>Phụ trách: F04 biến thể, F05 giỏ hàng, F06 MUA NGAY • 30 TC mỗi chức năng • F04 PASS 30/30 theo xác nhận; F05 và F06 chưa chạy</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
         <x:v>Phụ trách: F04, F05, F06  •  Case đầu tiên của mỗi chức năng: 30  •  Chưa chạy, chưa xác minh UI</x:v>
@@ -8494,14 +8514,14 @@
       </x:c>
       <x:c r="D3" s="32" t="n">
         <x:f>COUNTIF(M6:M95,"PASS")+COUNTIF(M6:M95,"FAIL")+COUNTIF(M6:M95,"BLOCKED")</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E3" s="32" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F3" s="32" t="n">
         <x:f>COUNTIF(M6:M95,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G3" s="32" t="str">
         <x:v>FAIL</x:v>
@@ -8515,7 +8535,7 @@
       </x:c>
       <x:c r="J3" s="32" t="n">
         <x:f>COUNTIF(O6:O95,"Đã xác minh")</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K3" s="32" t="str">
         <x:v>BLOCKED</x:v>
@@ -8615,15 +8635,17 @@
       <x:c r="K6" s="26" t="str">
         <x:v>Tên biến thể, giá và lựa chọn hiện hành đồng bộ.</x:v>
       </x:c>
-      <x:c r="L6" s="26"/>
+      <x:c r="L6" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M6" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N6" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O6" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P6" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8669,15 +8691,17 @@
       <x:c r="K7" s="26" t="str">
         <x:v>Tên biến thể, giá và lựa chọn hiện hành đồng bộ.</x:v>
       </x:c>
-      <x:c r="L7" s="26"/>
+      <x:c r="L7" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M7" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O7" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P7" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8723,15 +8747,17 @@
       <x:c r="K8" s="26" t="str">
         <x:v>Tên biến thể, giá và lựa chọn hiện hành đồng bộ.</x:v>
       </x:c>
-      <x:c r="L8" s="26"/>
+      <x:c r="L8" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M8" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N8" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O8" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P8" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8777,15 +8803,17 @@
       <x:c r="K9" s="26" t="str">
         <x:v>Tên biến thể, giá và lựa chọn hiện hành đồng bộ.</x:v>
       </x:c>
-      <x:c r="L9" s="26"/>
+      <x:c r="L9" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M9" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N9" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O9" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P9" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8831,15 +8859,17 @@
       <x:c r="K10" s="26" t="str">
         <x:v>Tên biến thể, giá và lựa chọn hiện hành đồng bộ.</x:v>
       </x:c>
-      <x:c r="L10" s="26"/>
+      <x:c r="L10" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M10" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N10" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O10" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P10" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8885,15 +8915,17 @@
       <x:c r="K11" s="26" t="str">
         <x:v>Màu đã chọn hiển thị đúng; ảnh/tên SKU phù hợp nếu hệ thống quy định.</x:v>
       </x:c>
-      <x:c r="L11" s="26"/>
+      <x:c r="L11" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M11" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N11" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O11" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P11" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8939,15 +8971,17 @@
       <x:c r="K12" s="26" t="str">
         <x:v>Màu đã chọn hiển thị đúng; ảnh/tên SKU phù hợp nếu hệ thống quy định.</x:v>
       </x:c>
-      <x:c r="L12" s="26"/>
+      <x:c r="L12" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M12" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N12" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O12" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P12" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -8993,15 +9027,17 @@
       <x:c r="K13" s="26" t="str">
         <x:v>Màu đã chọn hiển thị đúng; ảnh/tên SKU phù hợp nếu hệ thống quy định.</x:v>
       </x:c>
-      <x:c r="L13" s="26"/>
+      <x:c r="L13" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M13" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N13" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O13" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P13" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9047,15 +9083,17 @@
       <x:c r="K14" s="26" t="str">
         <x:v>Màu đã chọn hiển thị đúng; ảnh/tên SKU phù hợp nếu hệ thống quy định.</x:v>
       </x:c>
-      <x:c r="L14" s="26"/>
+      <x:c r="L14" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M14" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N14" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O14" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P14" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9101,15 +9139,17 @@
       <x:c r="K15" s="26" t="str">
         <x:v>Màu đã chọn hiển thị đúng; ảnh/tên SKU phù hợp nếu hệ thống quy định.</x:v>
       </x:c>
-      <x:c r="L15" s="26"/>
+      <x:c r="L15" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M15" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N15" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O15" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P15" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9155,15 +9195,17 @@
       <x:c r="K16" s="26" t="str">
         <x:v>Hệ thống giữ tổ hợp hợp lệ, không chọn SKU không tồn tại.</x:v>
       </x:c>
-      <x:c r="L16" s="26"/>
+      <x:c r="L16" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M16" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N16" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O16" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P16" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9209,15 +9251,17 @@
       <x:c r="K17" s="26" t="str">
         <x:v>Hệ thống giữ tổ hợp hợp lệ, không chọn SKU không tồn tại.</x:v>
       </x:c>
-      <x:c r="L17" s="26"/>
+      <x:c r="L17" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M17" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N17" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O17" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P17" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9263,15 +9307,17 @@
       <x:c r="K18" s="26" t="str">
         <x:v>Hệ thống giữ tổ hợp hợp lệ, không chọn SKU không tồn tại.</x:v>
       </x:c>
-      <x:c r="L18" s="26"/>
+      <x:c r="L18" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M18" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N18" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O18" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P18" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9317,15 +9363,17 @@
       <x:c r="K19" s="26" t="str">
         <x:v>Hệ thống giữ tổ hợp hợp lệ, không chọn SKU không tồn tại.</x:v>
       </x:c>
-      <x:c r="L19" s="26"/>
+      <x:c r="L19" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M19" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N19" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O19" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P19" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9371,15 +9419,17 @@
       <x:c r="K20" s="26" t="str">
         <x:v>Hệ thống giữ tổ hợp hợp lệ, không chọn SKU không tồn tại.</x:v>
       </x:c>
-      <x:c r="L20" s="26"/>
+      <x:c r="L20" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M20" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N20" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O20" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P20" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9425,15 +9475,17 @@
       <x:c r="K21" s="26" t="str">
         <x:v>Giá và chương trình hiển thị đúng với biến thể đang chọn.</x:v>
       </x:c>
-      <x:c r="L21" s="26"/>
+      <x:c r="L21" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M21" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N21" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O21" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P21" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9479,15 +9531,17 @@
       <x:c r="K22" s="26" t="str">
         <x:v>Giá và chương trình hiển thị đúng với biến thể đang chọn.</x:v>
       </x:c>
-      <x:c r="L22" s="26"/>
+      <x:c r="L22" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M22" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N22" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O22" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P22" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9533,15 +9587,17 @@
       <x:c r="K23" s="26" t="str">
         <x:v>Giá và chương trình hiển thị đúng với biến thể đang chọn.</x:v>
       </x:c>
-      <x:c r="L23" s="26"/>
+      <x:c r="L23" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M23" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N23" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O23" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P23" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9587,15 +9643,17 @@
       <x:c r="K24" s="26" t="str">
         <x:v>Giá và chương trình hiển thị đúng với biến thể đang chọn.</x:v>
       </x:c>
-      <x:c r="L24" s="26"/>
+      <x:c r="L24" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M24" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N24" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O24" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P24" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9641,15 +9699,17 @@
       <x:c r="K25" s="26" t="str">
         <x:v>Giá và chương trình hiển thị đúng với biến thể đang chọn.</x:v>
       </x:c>
-      <x:c r="L25" s="26"/>
+      <x:c r="L25" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M25" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N25" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O25" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P25" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9695,15 +9755,17 @@
       <x:c r="K26" s="26" t="str">
         <x:v>CTA và thông tin tồn kho tương thích biến thể; không mua biến thể hết hàng.</x:v>
       </x:c>
-      <x:c r="L26" s="26"/>
+      <x:c r="L26" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M26" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N26" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O26" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P26" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9749,15 +9811,17 @@
       <x:c r="K27" s="26" t="str">
         <x:v>CTA và thông tin tồn kho tương thích biến thể; không mua biến thể hết hàng.</x:v>
       </x:c>
-      <x:c r="L27" s="26"/>
+      <x:c r="L27" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M27" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N27" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O27" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P27" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9803,15 +9867,17 @@
       <x:c r="K28" s="26" t="str">
         <x:v>CTA và thông tin tồn kho tương thích biến thể; không mua biến thể hết hàng.</x:v>
       </x:c>
-      <x:c r="L28" s="26"/>
+      <x:c r="L28" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M28" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N28" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O28" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P28" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9857,15 +9923,17 @@
       <x:c r="K29" s="26" t="str">
         <x:v>CTA và thông tin tồn kho tương thích biến thể; không mua biến thể hết hàng.</x:v>
       </x:c>
-      <x:c r="L29" s="26"/>
+      <x:c r="L29" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M29" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N29" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O29" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P29" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9911,15 +9979,17 @@
       <x:c r="K30" s="26" t="str">
         <x:v>CTA và thông tin tồn kho tương thích biến thể; không mua biến thể hết hàng.</x:v>
       </x:c>
-      <x:c r="L30" s="26"/>
+      <x:c r="L30" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M30" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N30" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O30" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P30" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -9965,15 +10035,17 @@
       <x:c r="K31" s="26" t="str">
         <x:v>Biến thể đã chọn được truyền đúng đến bước tiếp theo.</x:v>
       </x:c>
-      <x:c r="L31" s="26"/>
+      <x:c r="L31" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M31" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N31" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O31" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P31" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -10019,15 +10091,17 @@
       <x:c r="K32" s="26" t="str">
         <x:v>Biến thể đã chọn được truyền đúng đến bước tiếp theo.</x:v>
       </x:c>
-      <x:c r="L32" s="26"/>
+      <x:c r="L32" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M32" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N32" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O32" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P32" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -10073,15 +10147,17 @@
       <x:c r="K33" s="26" t="str">
         <x:v>Biến thể đã chọn được truyền đúng đến bước tiếp theo.</x:v>
       </x:c>
-      <x:c r="L33" s="26"/>
+      <x:c r="L33" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M33" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N33" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O33" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P33" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -10127,15 +10203,17 @@
       <x:c r="K34" s="26" t="str">
         <x:v>Biến thể đã chọn được truyền đúng đến bước tiếp theo.</x:v>
       </x:c>
-      <x:c r="L34" s="26"/>
+      <x:c r="L34" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M34" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N34" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O34" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P34" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -10181,15 +10259,17 @@
       <x:c r="K35" s="26" t="str">
         <x:v>Biến thể đã chọn được truyền đúng đến bước tiếp theo.</x:v>
       </x:c>
-      <x:c r="L35" s="26"/>
+      <x:c r="L35" s="26" t="str">
+        <x:v>Đạt theo kết quả chạy Playwright TV2 đã xác nhận (30/30); xem ASM7 F04.</x:v>
+      </x:c>
       <x:c r="M35" s="30" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N35" s="30" t="str">
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O35" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã xác minh</x:v>
       </x:c>
       <x:c r="P35" s="26" t="str">
         <x:v>Cần chọn model có đủ biến thể để chạy tất cả tình huống.</x:v>
@@ -11235,7 +11315,7 @@
         <x:v>Quản lý giỏ hàng</x:v>
       </x:c>
       <x:c r="D55" s="26" t="str">
-        <x:v>Tính toán: Có ưu đãi mua kèm</x:v>
+        <x:v>Tính toán: Cập nhật tổng tiền sau khi xóa một trong hai mẫu</x:v>
       </x:c>
       <x:c r="E55" s="30" t="str">
         <x:v>Boundary</x:v>
@@ -11247,19 +11327,19 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="H55" s="26" t="str">
-        <x:v>Sản phẩm còn hàng; kiểm tra giỏ hàng khách vãng lai; không tạo đơn thật.</x:v>
+        <x:v>Giỏ có hai sản phẩm khác biến thể (Titan Xanh và Titan Đen); cả hai đang còn hàng. Không xác nhận đơn.</x:v>
       </x:c>
       <x:c r="I55" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Sản phẩm còn hàng; kiểm tra giỏ hàng khách vãng lai; không tạo đơn thật.
-3. Tương tác giỏ và đối chiếu số tiền; tình huống: Có ưu đãi mua kèm.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html; thêm Titan Xanh và Titan Đen vào giỏ qua nút xe đẩy.
+2. Mở giỏ, ghi giá và tổng tiền đang hiển thị.
+3. Xóa dòng Titan Đen theo điều khiển xóa của giỏ.
+4. Kiểm tra chỉ còn Titan Xanh; thành tiền giảm đúng giá dòng đã xóa, không đặt đơn.</x:v>
       </x:c>
       <x:c r="J55" s="26" t="str">
-        <x:v>Có ưu đãi mua kèm  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Samsung S25 Ultra 256GB Titan Xanh x1; Titan Đen x1; xóa Titan Đen</x:v>
       </x:c>
       <x:c r="K55" s="26" t="str">
-        <x:v>Thành tiền và tổng tiền phù hợp đơn giá, số lượng và ưu đãi công bố.</x:v>
+        <x:v>Chỉ còn Titan Xanh x1; tổng giỏ bằng giá thực tế của sản phẩm còn lại, không tính sản phẩm đã xóa.</x:v>
       </x:c>
       <x:c r="L55" s="26"/>
       <x:c r="M55" s="30" t="str">
@@ -11272,7 +11352,7 @@
         <x:v>Cần xác minh</x:v>
       </x:c>
       <x:c r="P55" s="26" t="str">
-        <x:v>Chỉ dùng giỏ và bước trước khi đặt hàng.</x:v>
+        <x:v>Thao tác chỉ trong giỏ; không yêu cầu chương trình ưu đãi riêng.</x:v>
       </x:c>
       <x:c r="Q55" s="26" t="str">
         <x:v>https://didongviet.vn/</x:v>
@@ -11826,10 +11906,10 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C66" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D66" s="26" t="str">
-        <x:v>Hiển thị gói mua kèm: Một gói mặc định</x:v>
+        <x:v>Mở luồng MUA NGAY cho Titan Xanh 256GB</x:v>
       </x:c>
       <x:c r="E66" s="30" t="str">
         <x:v>Positive</x:v>
@@ -11841,35 +11921,36 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="H66" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Từ trang mới, chọn 256GB và màu Titan Xanh; đảm bảo nút MUA NGAY khả dụng; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I66" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Mở vùng mua kèm trên trang chi tiết; tình huống: Một gói mặc định.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Từ trang mới, chọn 256GB và màu Titan Xanh; đảm bảo nút MUA NGAY khả dụng.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Ghi nhận tên, màu, dung lượng rồi bấm MUA NGAY đúng một lần.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J66" s="26" t="str">
-        <x:v>Một gói mặc định  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; số lượng ban đầu 1</x:v>
       </x:c>
       <x:c r="K66" s="26" t="str">
-        <x:v>Gói, tên hàng kèm và giá đúng theo thông tin niêm yết.</x:v>
+        <x:v>Đi đến bước mua hàng có liên quan đúng Galaxy S25 Ultra 256GB Titan Xanh; không tạo đơn thực tế; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L66" s="26"/>
       <x:c r="M66" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N66" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O66" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P66" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q66" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="69" customHeight="1">
@@ -11880,50 +11961,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C67" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D67" s="26" t="str">
-        <x:v>Hiển thị gói mua kèm: Gói có giá giảm</x:v>
+        <x:v>Mở luồng MUA NGAY cho Titan Đen 256GB</x:v>
       </x:c>
       <x:c r="E67" s="30" t="str">
         <x:v>Positive</x:v>
       </x:c>
       <x:c r="F67" s="30" t="str">
-        <x:v>Equivalence Partitioning</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G67" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H67" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chọn màu Titan Đen, phiên bản 256GB đang bán; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I67" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Mở vùng mua kèm trên trang chi tiết; tình huống: Gói có giá giảm.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chọn màu Titan Đen, phiên bản 256GB đang bán.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY và đối chiếu màu sản phẩm ở luồng mua.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J67" s="26" t="str">
-        <x:v>Gói có giá giảm  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Đen</x:v>
       </x:c>
       <x:c r="K67" s="26" t="str">
-        <x:v>Gói, tên hàng kèm và giá đúng theo thông tin niêm yết.</x:v>
+        <x:v>Không tự chuyển thành màu Titan Xanh/Bạc; màu được chọn phải giữ đúng nếu có phần tóm tắt; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L67" s="26"/>
       <x:c r="M67" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N67" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O67" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P67" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q67" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="69" customHeight="1">
@@ -11934,10 +12016,10 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C68" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D68" s="26" t="str">
-        <x:v>Hiển thị gói mua kèm: Gói gồm 2 món</x:v>
+        <x:v>Mở luồng MUA NGAY cho màu Bạc 256GB</x:v>
       </x:c>
       <x:c r="E68" s="30" t="str">
         <x:v>Positive</x:v>
@@ -11949,35 +12031,36 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="H68" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chọn màu Bạc, 256GB đang có thể mua; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I68" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Mở vùng mua kèm trên trang chi tiết; tình huống: Gói gồm 2 món.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chọn màu Bạc, 256GB đang có thể mua.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY, đối chiếu sản phẩm/màu trên màn hình kế tiếp.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J68" s="26" t="str">
-        <x:v>Gói gồm 2 món  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Bạc</x:v>
       </x:c>
       <x:c r="K68" s="26" t="str">
-        <x:v>Gói, tên hàng kèm và giá đúng theo thông tin niêm yết.</x:v>
+        <x:v>Đi đúng luồng mua của màu Bạc, không lấy biến thể khác; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L68" s="26"/>
       <x:c r="M68" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N68" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O68" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P68" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q68" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="69" customHeight="1">
@@ -11988,10 +12071,10 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C69" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D69" s="26" t="str">
-        <x:v>Hiển thị gói mua kèm: Gói có phụ kiện</x:v>
+        <x:v>Mở luồng MUA NGAY cho Xám Titan 256GB</x:v>
       </x:c>
       <x:c r="E69" s="30" t="str">
         <x:v>Positive</x:v>
@@ -12003,35 +12086,36 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="H69" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chọn Xám Titan và 256GB; kiểm tra nút đang bật; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I69" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Mở vùng mua kèm trên trang chi tiết; tình huống: Gói có phụ kiện.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chọn Xám Titan và 256GB; kiểm tra nút đang bật.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY, đọc tên sản phẩm và thông tin được mang sang.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J69" s="26" t="str">
-        <x:v>Gói có phụ kiện  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Xám Titan</x:v>
       </x:c>
       <x:c r="K69" s="26" t="str">
-        <x:v>Gói, tên hàng kèm và giá đúng theo thông tin niêm yết.</x:v>
+        <x:v>Biến thể Xám Titan được bảo toàn; luồng mua hiển thị hợp lệ; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L69" s="26"/>
       <x:c r="M69" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N69" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O69" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P69" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q69" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="69" customHeight="1">
@@ -12042,50 +12126,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C70" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D70" s="26" t="str">
-        <x:v>Hiển thị gói mua kèm: Gói có quà tặng nếu có</x:v>
+        <x:v>Nút MUA NGAY và biểu tượng giỏ là hai hành động khác nhau</x:v>
       </x:c>
       <x:c r="E70" s="30" t="str">
         <x:v>Positive</x:v>
       </x:c>
       <x:c r="F70" s="30" t="str">
-        <x:v>Equivalence Partitioning</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G70" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H70" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Có trang chi tiết với cả nút MUA NGAY và biểu tượng xe đẩy viền đỏ; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I70" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Mở vùng mua kèm trên trang chi tiết; tình huống: Gói có quà tặng nếu có.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Có trang chi tiết với cả nút MUA NGAY và biểu tượng xe đẩy viền đỏ.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Ghi lại hai điều khiển; bấm riêng nút MUA NGAY, quan sát màn hình chuyển đến.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J70" s="26" t="str">
-        <x:v>Gói có quà tặng nếu có  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; CTA = MUA NGAY</x:v>
       </x:c>
       <x:c r="K70" s="26" t="str">
-        <x:v>Gói, tên hàng kèm và giá đúng theo thông tin niêm yết.</x:v>
+        <x:v>Nhấn MUA NGAY đưa vào luồng mua, không chỉ hiển thị thông báo thêm giỏ như nút xe đẩy; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L70" s="26"/>
       <x:c r="M70" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N70" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O70" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P70" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q70" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="69" customHeight="1">
@@ -12096,50 +12181,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C71" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D71" s="26" t="str">
-        <x:v>Chọn và bỏ chọn: Chọn 1 món kèm</x:v>
+        <x:v>Đổi Titan Xanh sang Titan Đen trước MUA NGAY</x:v>
       </x:c>
       <x:c r="E71" s="30" t="str">
-        <x:v>Combination</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F71" s="30" t="str">
-        <x:v>Decision Table</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G71" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H71" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chọn 256GB Titan Xanh rồi chuyển sang Titan Đen; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I71" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Bật/tắt lựa chọn hàng mua kèm; tình huống: Chọn 1 món kèm.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chọn 256GB Titan Xanh rồi chuyển sang Titan Đen.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Sau khi UI cập nhật xong, nhấn MUA NGAY và so sánh biến thể cuối.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J71" s="26" t="str">
-        <x:v>Chọn 1 món kèm  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh → Titan Đen</x:v>
       </x:c>
       <x:c r="K71" s="26" t="str">
-        <x:v>Trạng thái chọn và số tiền cộng thêm cập nhật đúng.</x:v>
+        <x:v>Luồng mua sử dụng Titan Đen mới nhất, không giữ màu trước đó; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L71" s="26"/>
       <x:c r="M71" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N71" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O71" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P71" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q71" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="69" customHeight="1">
@@ -12150,50 +12236,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C72" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D72" s="26" t="str">
-        <x:v>Chọn và bỏ chọn: Bỏ 1 món kèm</x:v>
+        <x:v>Đổi Titan Đen sang màu Bạc trước MUA NGAY</x:v>
       </x:c>
       <x:c r="E72" s="30" t="str">
-        <x:v>Combination</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F72" s="30" t="str">
-        <x:v>Decision Table</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G72" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H72" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chọn 256GB Titan Đen rồi chuyển màu Bạc; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I72" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Bật/tắt lựa chọn hàng mua kèm; tình huống: Bỏ 1 món kèm.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chọn 256GB Titan Đen rồi chuyển màu Bạc.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Nhấn MUA NGAY và đối chiếu tên/màu trên màn hình kế tiếp.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J72" s="26" t="str">
-        <x:v>Bỏ 1 món kèm  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Đen → Bạc</x:v>
       </x:c>
       <x:c r="K72" s="26" t="str">
-        <x:v>Trạng thái chọn và số tiền cộng thêm cập nhật đúng.</x:v>
+        <x:v>Giữ đúng Bạc là màu cuối cùng; không xảy ra dữ liệu cũ; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L72" s="26"/>
       <x:c r="M72" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N72" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O72" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P72" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q72" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="69" customHeight="1">
@@ -12204,50 +12291,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C73" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D73" s="26" t="str">
-        <x:v>Chọn và bỏ chọn: Chọn 2 món kèm nếu hỗ trợ</x:v>
+        <x:v>Đổi Bạc sang Xám Titan trước MUA NGAY</x:v>
       </x:c>
       <x:c r="E73" s="30" t="str">
-        <x:v>Combination</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F73" s="30" t="str">
-        <x:v>Decision Table</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G73" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H73" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Đang ở 256GB Bạc, chuyển sang Xám Titan; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I73" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Bật/tắt lựa chọn hàng mua kèm; tình huống: Chọn 2 món kèm nếu hỗ trợ.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Đang ở 256GB Bạc, chuyển sang Xám Titan.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Nhấn MUA NGAY khi giá và biến thể đã tải xong.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J73" s="26" t="str">
-        <x:v>Chọn 2 món kèm nếu hỗ trợ  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Bạc → Xám Titan</x:v>
       </x:c>
       <x:c r="K73" s="26" t="str">
-        <x:v>Trạng thái chọn và số tiền cộng thêm cập nhật đúng.</x:v>
+        <x:v>Thông tin mua là Xám Titan chứ không phải màu Bạc ban đầu; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L73" s="26"/>
       <x:c r="M73" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N73" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O73" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P73" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q73" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="69" customHeight="1">
@@ -12258,34 +12346,35 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C74" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D74" s="26" t="str">
-        <x:v>Chọn và bỏ chọn: Bỏ tất cả</x:v>
+        <x:v>Chuyển từ 256GB sang 512GB rồi MUA NGAY</x:v>
       </x:c>
       <x:c r="E74" s="30" t="str">
-        <x:v>Combination</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="F74" s="30" t="str">
-        <x:v>Decision Table</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G74" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H74" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Trên trang có tùy chọn 512GB; biến thể này còn hàng và có nút MUA NGAY; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I74" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Bật/tắt lựa chọn hàng mua kèm; tình huống: Bỏ tất cả.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Trên trang có tùy chọn 512GB; biến thể này còn hàng và có nút MUA NGAY.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Chọn 512GB, ghi tên SKU/giá, sau đó nhấn MUA NGAY.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J74" s="26" t="str">
-        <x:v>Bỏ tất cả  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB → 512GB; Titan Xanh nếu khả dụng</x:v>
       </x:c>
       <x:c r="K74" s="26" t="str">
-        <x:v>Trạng thái chọn và số tiền cộng thêm cập nhật đúng.</x:v>
+        <x:v>Luồng mua là 512GB; không tự quay về 256GB. Nếu SKU không mua được thì ghi Blocked; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L74" s="26"/>
       <x:c r="M74" s="30" t="str">
@@ -12295,13 +12384,13 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="O74" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P74" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q74" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="69" customHeight="1">
@@ -12312,34 +12401,35 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C75" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D75" s="26" t="str">
-        <x:v>Chọn và bỏ chọn: Chọn lại sau khi bỏ</x:v>
+        <x:v>Từ 512GB quay về 256GB trước MUA NGAY</x:v>
       </x:c>
       <x:c r="E75" s="30" t="str">
-        <x:v>Combination</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="F75" s="30" t="str">
-        <x:v>Decision Table</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G75" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H75" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Đã điều hướng sang bản 512GB còn hàng, sau đó chọn lại 256GB; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I75" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Bật/tắt lựa chọn hàng mua kèm; tình huống: Chọn lại sau khi bỏ.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Đã điều hướng sang bản 512GB còn hàng, sau đó chọn lại 256GB.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY sau khi 256GB xuất hiện ổn định.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J75" s="26" t="str">
-        <x:v>Chọn lại sau khi bỏ  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>512GB → 256GB; Bạc nếu khả dụng</x:v>
       </x:c>
       <x:c r="K75" s="26" t="str">
-        <x:v>Trạng thái chọn và số tiền cộng thêm cập nhật đúng.</x:v>
+        <x:v>Luồng mua đúng 256GB, không mang thông tin 512GB còn lưu trong phiên; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L75" s="26"/>
       <x:c r="M75" s="30" t="str">
@@ -12349,13 +12439,13 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="O75" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P75" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q75" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="69" customHeight="1">
@@ -12366,34 +12456,35 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C76" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D76" s="26" t="str">
-        <x:v>Thay sản phẩm chính: Đổi màu máy</x:v>
+        <x:v>Chọn 1TB rồi MUA NGAY khi sản phẩm khả dụng</x:v>
       </x:c>
       <x:c r="E76" s="30" t="str">
-        <x:v>State</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="F76" s="30" t="str">
-        <x:v>State Transition</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G76" s="30" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H76" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Trang hiển thị bản 1TB, còn hàng và có nút MUA NGAY; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I76" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đổi phiên bản máy khi đang chọn mua kèm; tình huống: Đổi màu máy.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Trang hiển thị bản 1TB, còn hàng và có nút MUA NGAY.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Chọn 1TB; chờ cập nhật thông tin rồi bấm MUA NGAY.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J76" s="26" t="str">
-        <x:v>Đổi màu máy  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB → 1TB; màu có hàng</x:v>
       </x:c>
       <x:c r="K76" s="26" t="str">
-        <x:v>Ưu đãi/giá mua kèm cập nhật theo sản phẩm chính mới.</x:v>
+        <x:v>Nếu phiên bản 1TB mua được thì luồng mua giữ 1TB; nếu thiếu tồn kho, đánh dấu Blocked; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L76" s="26"/>
       <x:c r="M76" s="30" t="str">
@@ -12403,13 +12494,13 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="O76" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P76" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q76" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="69" customHeight="1">
@@ -12420,50 +12511,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C77" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D77" s="26" t="str">
-        <x:v>Thay sản phẩm chính: Đổi dung lượng</x:v>
+        <x:v>Chọn lại cùng màu trước khi MUA NGAY</x:v>
       </x:c>
       <x:c r="E77" s="30" t="str">
-        <x:v>State</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F77" s="30" t="str">
-        <x:v>State Transition</x:v>
+        <x:v>Boundary Value</x:v>
       </x:c>
       <x:c r="G77" s="30" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H77" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chọn 256GB Titan Xanh rồi bấm lại chính màu Titan Xanh; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I77" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đổi phiên bản máy khi đang chọn mua kèm; tình huống: Đổi dung lượng.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chọn 256GB Titan Xanh rồi bấm lại chính màu Titan Xanh.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY, so sánh SKU với giá trị trước và sau thao tác lặp.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J77" s="26" t="str">
-        <x:v>Đổi dung lượng  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh → Titan Xanh</x:v>
       </x:c>
       <x:c r="K77" s="26" t="str">
-        <x:v>Ưu đãi/giá mua kèm cập nhật theo sản phẩm chính mới.</x:v>
+        <x:v>Không bị reset sang màu khác, không tạo hai dòng sản phẩm vì bấm lại màu; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L77" s="26"/>
       <x:c r="M77" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N77" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O77" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P77" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q77" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="69" customHeight="1">
@@ -12474,50 +12566,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C78" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D78" s="26" t="str">
-        <x:v>Thay sản phẩm chính: Đổi về cấu hình cũ</x:v>
+        <x:v>Đối chiếu giá Titan Xanh trước và sau MUA NGAY</x:v>
       </x:c>
       <x:c r="E78" s="30" t="str">
-        <x:v>State</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F78" s="30" t="str">
-        <x:v>State Transition</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G78" s="30" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H78" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Mở 256GB Titan Xanh đang bán; ghi giá thực tế tại thời điểm chạy; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I78" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đổi phiên bản máy khi đang chọn mua kèm; tình huống: Đổi về cấu hình cũ.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Mở 256GB Titan Xanh đang bán; ghi giá thực tế tại thời điểm chạy.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY, kiểm tra giá hiển thị ở phần thông tin mua nếu trang có.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J78" s="26" t="str">
-        <x:v>Đổi về cấu hình cũ  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; giá ghi lúc chạy</x:v>
       </x:c>
       <x:c r="K78" s="26" t="str">
-        <x:v>Ưu đãi/giá mua kèm cập nhật theo sản phẩm chính mới.</x:v>
+        <x:v>Giá đơn vị/tạm tính phù hợp với giá hiện hành và điều kiện ưu đãi công bố; không dùng giá cố định; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L78" s="26"/>
       <x:c r="M78" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N78" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O78" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P78" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q78" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="69" customHeight="1">
@@ -12528,50 +12621,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C79" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D79" s="26" t="str">
-        <x:v>Thay sản phẩm chính: Đổi sang phiên bản đắt hơn</x:v>
+        <x:v>Đối chiếu giá Titan Đen trước và sau MUA NGAY</x:v>
       </x:c>
       <x:c r="E79" s="30" t="str">
-        <x:v>State</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F79" s="30" t="str">
-        <x:v>State Transition</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G79" s="30" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H79" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Mở 256GB Titan Đen; ghi giá bên cạnh màu/giá bán; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I79" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đổi phiên bản máy khi đang chọn mua kèm; tình huống: Đổi sang phiên bản đắt hơn.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Mở 256GB Titan Đen; ghi giá bên cạnh màu/giá bán.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY và đối chiếu giá tại bước tiếp theo.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J79" s="26" t="str">
-        <x:v>Đổi sang phiên bản đắt hơn  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Đen; giá ghi lúc chạy</x:v>
       </x:c>
       <x:c r="K79" s="26" t="str">
-        <x:v>Ưu đãi/giá mua kèm cập nhật theo sản phẩm chính mới.</x:v>
+        <x:v>Không lấy nhầm giá Titan Xanh cho Titan Đen; không tự nhân đôi số lượng; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L79" s="26"/>
       <x:c r="M79" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N79" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O79" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P79" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q79" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="69" customHeight="1">
@@ -12582,50 +12676,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C80" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D80" s="26" t="str">
-        <x:v>Thay sản phẩm chính: Đổi sang phiên bản hết hàng nếu có</x:v>
+        <x:v>Phân biệt giá bán hiện tại với giá gạch</x:v>
       </x:c>
       <x:c r="E80" s="30" t="str">
-        <x:v>State</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F80" s="30" t="str">
-        <x:v>State Transition</x:v>
+        <x:v>Boundary Value</x:v>
       </x:c>
       <x:c r="G80" s="30" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H80" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Trang sản phẩm có thể hiển thị giá bán và giá gốc gạch ngang; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I80" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đổi phiên bản máy khi đang chọn mua kèm; tình huống: Đổi sang phiên bản hết hàng nếu có.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Trang sản phẩm có thể hiển thị giá bán và giá gốc gạch ngang.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Ghi cả hai loại giá, bấm MUA NGAY và kiểm tra số tiền có tính trên đơn.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J80" s="26" t="str">
-        <x:v>Đổi sang phiên bản hết hàng nếu có  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; giá bán/giá gạch</x:v>
       </x:c>
       <x:c r="K80" s="26" t="str">
-        <x:v>Ưu đãi/giá mua kèm cập nhật theo sản phẩm chính mới.</x:v>
+        <x:v>Số tiền mua không sử dụng nhầm giá gạch; ưu đãi chỉ tính khi có điều kiện hợp lệ; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L80" s="26"/>
       <x:c r="M80" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N80" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O80" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P80" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q80" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="69" customHeight="1">
@@ -12636,50 +12731,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C81" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D81" s="26" t="str">
-        <x:v>Tính giá combo: Chỉ sản phẩm chính</x:v>
+        <x:v>Kiểm tra số lượng mặc định trong luồng MUA NGAY</x:v>
       </x:c>
       <x:c r="E81" s="30" t="str">
-        <x:v>Boundary</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F81" s="30" t="str">
-        <x:v>Boundary Value Analysis</x:v>
+        <x:v>Boundary Value</x:v>
       </x:c>
       <x:c r="G81" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H81" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Phiên làm việc mới, chưa có thao tác thay số lượng ở luồng mua; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I81" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đối chiếu số tiền khi bật ưu đãi mua kèm; tình huống: Chỉ sản phẩm chính.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Phiên làm việc mới, chưa có thao tác thay số lượng ở luồng mua.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Chọn 256GB màu Bạc; bấm MUA NGAY rồi đọc số lượng hiển thị nếu có.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J81" s="26" t="str">
-        <x:v>Chỉ sản phẩm chính  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Bạc; một lần nhấn</x:v>
       </x:c>
       <x:c r="K81" s="26" t="str">
-        <x:v>Giá combo bằng giá thành phần sau các quy tắc giảm giá được công bố.</x:v>
+        <x:v>Chỉ một máy theo thao tác MUA NGAY một lần; không tự phát sinh số lượng 2 hoặc nhiều dòng giống nhau; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L81" s="26"/>
       <x:c r="M81" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N81" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O81" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P81" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q81" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="69" customHeight="1">
@@ -12690,50 +12786,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C82" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D82" s="26" t="str">
-        <x:v>Tính giá combo: Chính + 1 món</x:v>
+        <x:v>Kiểm tra thông tin tên sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="E82" s="30" t="str">
-        <x:v>Boundary</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F82" s="30" t="str">
-        <x:v>Boundary Value Analysis</x:v>
+        <x:v>Equivalence Partitioning</x:v>
       </x:c>
       <x:c r="G82" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H82" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Trang chi tiết hiển thị Galaxy S25 Ultra 256GB Chính Hãng; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I82" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đối chiếu số tiền khi bật ưu đãi mua kèm; tình huống: Chính + 1 món.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Trang chi tiết hiển thị Galaxy S25 Ultra 256GB Chính Hãng.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY, tìm tên sản phẩm ở tóm tắt/trạng thái được chuyển đến.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J82" s="26" t="str">
-        <x:v>Chính + 1 món  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Samsung Galaxy S25 Ultra 256GB Chính Hãng</x:v>
       </x:c>
       <x:c r="K82" s="26" t="str">
-        <x:v>Giá combo bằng giá thành phần sau các quy tắc giảm giá được công bố.</x:v>
+        <x:v>Không chuyển sang sản phẩm Samsung khác; thông tin sản phẩm phải nhất quán; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L82" s="26"/>
       <x:c r="M82" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N82" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O82" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P82" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q82" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="69" customHeight="1">
@@ -12744,34 +12841,35 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C83" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D83" s="26" t="str">
-        <x:v>Tính giá combo: Chính + 2 món</x:v>
+        <x:v>Ưu đãi thay đổi theo ngày không làm sai thông tin SKU</x:v>
       </x:c>
       <x:c r="E83" s="30" t="str">
-        <x:v>Boundary</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="F83" s="30" t="str">
-        <x:v>Boundary Value Analysis</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G83" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H83" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Giá/ưu đãi có thể thay đổi; ghi nhận giá tại thời điểm chạy trước khi bấm; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I83" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đối chiếu số tiền khi bật ưu đãi mua kèm; tình huống: Chính + 2 món.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Giá/ưu đãi có thể thay đổi; ghi nhận giá tại thời điểm chạy trước khi bấm.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Chọn Titan Xanh, bấm MUA NGAY, đối chiếu giá cuối với điều kiện ưu đãi đang áp dụng.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J83" s="26" t="str">
-        <x:v>Chính + 2 món  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; giá tại thời điểm test</x:v>
       </x:c>
       <x:c r="K83" s="26" t="str">
-        <x:v>Giá combo bằng giá thành phần sau các quy tắc giảm giá được công bố.</x:v>
+        <x:v>Giá và SKU nhất quán, không cam kết giữ giá cũ nếu chương trình đã hết hạn; chỉ yêu cầu minh bạch chênh lệch; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L83" s="26"/>
       <x:c r="M83" s="30" t="str">
@@ -12781,13 +12879,13 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="O83" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P83" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q83" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="69" customHeight="1">
@@ -12798,50 +12896,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C84" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D84" s="26" t="str">
-        <x:v>Tính giá combo: Bỏ 1 trong 2 món</x:v>
+        <x:v>MUA NGAY khi giỏ hiện đang trống</x:v>
       </x:c>
       <x:c r="E84" s="30" t="str">
-        <x:v>Boundary</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F84" s="30" t="str">
-        <x:v>Boundary Value Analysis</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G84" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H84" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Khởi tạo phiên sạch; xác minh giỏ chưa chứa sản phẩm; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I84" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đối chiếu số tiền khi bật ưu đãi mua kèm; tình huống: Bỏ 1 trong 2 món.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Khởi tạo phiên sạch; xác minh giỏ chưa chứa sản phẩm.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Mở S25 Ultra 256GB Titan Xanh, bấm MUA NGAY và quan sát luồng tiếp theo.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J84" s="26" t="str">
-        <x:v>Bỏ 1 trong 2 món  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Giỏ trống; Titan Xanh; MUA NGAY</x:v>
       </x:c>
       <x:c r="K84" s="26" t="str">
-        <x:v>Giá combo bằng giá thành phần sau các quy tắc giảm giá được công bố.</x:v>
+        <x:v>Không bắt người dùng nhấn biểu tượng xe đẩy trước mới được MUA NGAY; luồng mua xuất hiện hợp lệ; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L84" s="26"/>
       <x:c r="M84" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N84" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O84" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Cần kiểm tra dữ liệu</x:v>
       </x:c>
       <x:c r="P84" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q84" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="69" customHeight="1">
@@ -12852,50 +12951,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C85" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D85" s="26" t="str">
-        <x:v>Tính giá combo: Ưu đãi hết hạn nếu có dữ liệu</x:v>
+        <x:v>MUA NGAY khi giỏ đã chứa S25 Ultra màu khác</x:v>
       </x:c>
       <x:c r="E85" s="30" t="str">
-        <x:v>Boundary</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F85" s="30" t="str">
-        <x:v>Boundary Value Analysis</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G85" s="30" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H85" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chuẩn bị giỏ có 1 S25 Ultra 256GB Titan Đen bằng nút xe đẩy; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I85" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Đối chiếu số tiền khi bật ưu đãi mua kèm; tình huống: Ưu đãi hết hạn nếu có dữ liệu.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chuẩn bị giỏ có 1 S25 Ultra 256GB Titan Đen bằng nút xe đẩy.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Quay lại trang sản phẩm, chọn Titan Xanh và nhấn MUA NGAY; so sánh thông tin đang mua.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J85" s="26" t="str">
-        <x:v>Ưu đãi hết hạn nếu có dữ liệu  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Giỏ: Titan Đen x1; MUA NGAY: Titan Xanh</x:v>
       </x:c>
       <x:c r="K85" s="26" t="str">
-        <x:v>Giá combo bằng giá thành phần sau các quy tắc giảm giá được công bố.</x:v>
+        <x:v>Sản phẩm đang MUA NGAY là Titan Xanh; không tự chuyển thành Titan Đen do giỏ đã có hàng; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L85" s="26"/>
       <x:c r="M85" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N85" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O85" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Cần kiểm tra dữ liệu</x:v>
       </x:c>
       <x:c r="P85" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q85" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="69" customHeight="1">
@@ -12906,50 +13006,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C86" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D86" s="26" t="str">
-        <x:v>Ràng buộc điều kiện: Không chọn máy chính</x:v>
+        <x:v>MUA NGAY khi giỏ có cùng SKU</x:v>
       </x:c>
       <x:c r="E86" s="30" t="str">
-        <x:v>Negative</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F86" s="30" t="str">
-        <x:v>Negative / Combination</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G86" s="30" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="H86" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Chuẩn bị giỏ có S25 Ultra 256GB Titan Xanh x1; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I86" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Kiểm tra điều kiện được hưởng ưu đãi mua kèm; tình huống: Không chọn máy chính.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Chuẩn bị giỏ có S25 Ultra 256GB Titan Xanh x1.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Quay lại trang chi tiết, bấm MUA NGAY đúng một lần; theo dõi bước tiếp.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J86" s="26" t="str">
-        <x:v>Không chọn máy chính  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Giỏ: Titan Xanh x1; MUA NGAY Titan Xanh</x:v>
       </x:c>
       <x:c r="K86" s="26" t="str">
-        <x:v>Hệ thống không áp giá ưu đãi cho trường hợp không đủ điều kiện.</x:v>
+        <x:v>Màn hình chuyển tiếp phản ánh thao tác mua hiện tại; không tự phát sinh đơn hàng thành công hoặc nhân đôi không chủ đích; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L86" s="26"/>
       <x:c r="M86" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N86" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O86" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Cần kiểm tra dữ liệu</x:v>
       </x:c>
       <x:c r="P86" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q86" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="69" customHeight="1">
@@ -12960,50 +13061,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C87" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D87" s="26" t="str">
-        <x:v>Ràng buộc điều kiện: Đổi sang SKU không áp dụng</x:v>
+        <x:v>MUA NGAY sau khi đã thêm vào giỏ rồi quay lại sản phẩm</x:v>
       </x:c>
       <x:c r="E87" s="30" t="str">
-        <x:v>Negative</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F87" s="30" t="str">
-        <x:v>Negative / Combination</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G87" s="30" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="H87" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Đã thêm S25 Ultra 256GB màu Bạc vào giỏ, tiếp đó quay về sản phẩm; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I87" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Kiểm tra điều kiện được hưởng ưu đãi mua kèm; tình huống: Đổi sang SKU không áp dụng.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Đã thêm S25 Ultra 256GB màu Bạc vào giỏ, tiếp đó quay về sản phẩm.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Bấm MUA NGAY trên màu Bạc và quan sát điều hướng.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J87" s="26" t="str">
-        <x:v>Đổi sang SKU không áp dụng  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Đã thêm giỏ: Bạc x1; MUA NGAY: Bạc</x:v>
       </x:c>
       <x:c r="K87" s="26" t="str">
-        <x:v>Hệ thống không áp giá ưu đãi cho trường hợp không đủ điều kiện.</x:v>
+        <x:v>MUA NGAY hoạt động độc lập với thao tác mở giỏ; dẫn đến bước mua hợp lệ, không kích hoạt nút trả góp; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L87" s="26"/>
       <x:c r="M87" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N87" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O87" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Cần kiểm tra dữ liệu</x:v>
       </x:c>
       <x:c r="P87" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q87" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="69" customHeight="1">
@@ -13014,50 +13116,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C88" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D88" s="26" t="str">
-        <x:v>Ràng buộc điều kiện: Hết hàng mua kèm nếu có</x:v>
+        <x:v>MUA NGAY không tự kích hoạt trả góp 0%</x:v>
       </x:c>
       <x:c r="E88" s="30" t="str">
-        <x:v>Negative</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F88" s="30" t="str">
-        <x:v>Negative / Combination</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G88" s="30" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="H88" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Trang có hai nút Trả góp 0% và MUA NGAY cạnh nhau; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I88" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Kiểm tra điều kiện được hưởng ưu đãi mua kèm; tình huống: Hết hàng mua kèm nếu có.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Trang có hai nút Trả góp 0% và MUA NGAY cạnh nhau.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Chọn Titan Xanh, chỉ nhấn MUA NGAY, theo dõi giao diện điều hướng.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J88" s="26" t="str">
-        <x:v>Hết hàng mua kèm nếu có  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; nút MUA NGAY</x:v>
       </x:c>
       <x:c r="K88" s="26" t="str">
-        <x:v>Hệ thống không áp giá ưu đãi cho trường hợp không đủ điều kiện.</x:v>
+        <x:v>Không vào mặc định biểu mẫu đăng ký trả góp do nhầm vị trí CTA; hiển thị luồng mua thường; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L88" s="26"/>
       <x:c r="M88" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N88" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O88" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Cần kiểm tra dữ liệu</x:v>
       </x:c>
       <x:c r="P88" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q88" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="69" customHeight="1">
@@ -13068,50 +13171,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C89" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D89" s="26" t="str">
-        <x:v>Ràng buộc điều kiện: Món mua kèm trùng SKU chính</x:v>
+        <x:v>Quay lại trang sản phẩm từ luồng MUA NGAY</x:v>
       </x:c>
       <x:c r="E89" s="30" t="str">
-        <x:v>Negative</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F89" s="30" t="str">
-        <x:v>Negative / Combination</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G89" s="30" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="H89" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Mở luồng mua qua MUA NGAY; chưa nhập dữ liệu cá nhân; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I89" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Kiểm tra điều kiện được hưởng ưu đãi mua kèm; tình huống: Món mua kèm trùng SKU chính.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Mở luồng mua qua MUA NGAY; chưa nhập dữ liệu cá nhân.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Sử dụng nút Back của trình duyệt, đọc URL, tên máy và màu sản phẩm.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J89" s="26" t="str">
-        <x:v>Món mua kèm trùng SKU chính  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Bạc; Back</x:v>
       </x:c>
       <x:c r="K89" s="26" t="str">
-        <x:v>Hệ thống không áp giá ưu đãi cho trường hợp không đủ điều kiện.</x:v>
+        <x:v>Có thể trở về trang chi tiết an toàn; không có đơn đặt hàng được tạo chỉ từ thao tác Back; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L89" s="26"/>
       <x:c r="M89" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N89" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O89" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P89" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q89" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="69" customHeight="1">
@@ -13122,34 +13226,35 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C90" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D90" s="26" t="str">
-        <x:v>Ràng buộc điều kiện: Tối đa số món nếu có quy định</x:v>
+        <x:v>Tiếp tục bằng Forward sau khi Back</x:v>
       </x:c>
       <x:c r="E90" s="30" t="str">
-        <x:v>Negative</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="F90" s="30" t="str">
-        <x:v>Negative / Combination</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G90" s="30" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="H90" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Bắt đầu MUA NGAY cho Titan Xanh; thao tác Back về trang sản phẩm; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I90" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Kiểm tra điều kiện được hưởng ưu đãi mua kèm; tình huống: Tối đa số món nếu có quy định.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Bắt đầu MUA NGAY cho Titan Xanh; thao tác Back về trang sản phẩm.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Nhấn Forward; quan sát màn hình và trạng thái sản phẩm được mở lại.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J90" s="26" t="str">
-        <x:v>Tối đa số món nếu có quy định  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; Back → Forward</x:v>
       </x:c>
       <x:c r="K90" s="26" t="str">
-        <x:v>Hệ thống không áp giá ưu đãi cho trường hợp không đủ điều kiện.</x:v>
+        <x:v>Lịch sử điều hướng hợp lệ, không báo đặt hàng thành công hoặc tự xác nhận đơn; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L90" s="26"/>
       <x:c r="M90" s="30" t="str">
@@ -13159,13 +13264,13 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="O90" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P90" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q90" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="69" customHeight="1">
@@ -13176,50 +13281,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C91" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D91" s="26" t="str">
-        <x:v>Đồng bộ sang giỏ: Chính + 1 món vào giỏ</x:v>
+        <x:v>Tải lại trang sản phẩm trước khi nhấn MUA NGAY</x:v>
       </x:c>
       <x:c r="E91" s="30" t="str">
-        <x:v>Consistency</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F91" s="30" t="str">
-        <x:v>State / UI Consistency</x:v>
+        <x:v>State Transition</x:v>
       </x:c>
       <x:c r="G91" s="30" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H91" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Đang xem S25 Ultra 256GB Titan Đen, chưa bắt đầu mua; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I91" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Chuyển sản phẩm/gói đã chọn vào giỏ (không đặt hàng); tình huống: Chính + 1 món vào giỏ.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Đang xem S25 Ultra 256GB Titan Đen, chưa bắt đầu mua.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Refresh trang chi tiết; chọn lại Titan Đen nếu UI reset rồi nhấn MUA NGAY.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J91" s="26" t="str">
-        <x:v>Chính + 1 món vào giỏ  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Đen; Refresh → MUA NGAY</x:v>
       </x:c>
       <x:c r="K91" s="26" t="str">
-        <x:v>Giỏ phản ánh đúng món mua kèm, giá, số lượng và ưu đãi.</x:v>
+        <x:v>Luồng mua có đúng Titan Đen được chọn sau refresh; không mua nhầm SKU mặc định; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L91" s="26"/>
       <x:c r="M91" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N91" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O91" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Cần kiểm tra dữ liệu</x:v>
       </x:c>
       <x:c r="P91" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q91" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="69" customHeight="1">
@@ -13230,34 +13336,35 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C92" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D92" s="26" t="str">
-        <x:v>Đồng bộ sang giỏ: Chính + 2 món vào giỏ</x:v>
+        <x:v>Chỉ một lần chuyển luồng khi nhấn nhanh hai lần</x:v>
       </x:c>
       <x:c r="E92" s="30" t="str">
-        <x:v>Consistency</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="F92" s="30" t="str">
-        <x:v>State / UI Consistency</x:v>
+        <x:v>Boundary Value</x:v>
       </x:c>
       <x:c r="G92" s="30" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H92" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Có sản phẩm khả dụng; trình duyệt chưa vào luồng mua; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I92" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Chuyển sản phẩm/gói đã chọn vào giỏ (không đặt hàng); tình huống: Chính + 2 món vào giỏ.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Có sản phẩm khả dụng; trình duyệt chưa vào luồng mua.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Nhấn MUA NGAY hai lần nhanh trong UI nếu nút vẫn nhận; quan sát số lần mở luồng.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J92" s="26" t="str">
-        <x:v>Chính + 2 món vào giỏ  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; 2 clicks gần nhau</x:v>
       </x:c>
       <x:c r="K92" s="26" t="str">
-        <x:v>Giỏ phản ánh đúng món mua kèm, giá, số lượng và ưu đãi.</x:v>
+        <x:v>Không tạo đơn/luồng trùng lặp không chủ đích; nút có thể chặn nhấn lặp hoặc chuyển trang một lần; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L92" s="26"/>
       <x:c r="M92" s="30" t="str">
@@ -13267,13 +13374,13 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="O92" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P92" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q92" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="69" customHeight="1">
@@ -13284,50 +13391,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C93" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D93" s="26" t="str">
-        <x:v>Đồng bộ sang giỏ: Bỏ kèm trước khi thêm</x:v>
+        <x:v>Kiểm tra nút MUA NGAY ở kích thước desktop</x:v>
       </x:c>
       <x:c r="E93" s="30" t="str">
-        <x:v>Consistency</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F93" s="30" t="str">
-        <x:v>State / UI Consistency</x:v>
+        <x:v>Boundary Value</x:v>
       </x:c>
       <x:c r="G93" s="30" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H93" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Trình duyệt desktop viewport 1366 x 768; sản phẩm 256GB có thể mua; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I93" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Chuyển sản phẩm/gói đã chọn vào giỏ (không đặt hàng); tình huống: Bỏ kèm trước khi thêm.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Trình duyệt desktop viewport 1366 x 768; sản phẩm 256GB có thể mua.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Cuộn đến khối mua, nhấn MUA NGAY và quan sát điều hướng.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J93" s="26" t="str">
-        <x:v>Bỏ kèm trước khi thêm  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Desktop 1366×768; Titan Xanh</x:v>
       </x:c>
       <x:c r="K93" s="26" t="str">
-        <x:v>Giỏ phản ánh đúng món mua kèm, giá, số lượng và ưu đãi.</x:v>
+        <x:v>Nút hiển thị, bấm được, không bị che bởi lớp phủ; vào luồng mua đúng SKU; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L93" s="26"/>
       <x:c r="M93" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N93" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O93" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P93" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q93" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="69" customHeight="1">
@@ -13338,50 +13446,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C94" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D94" s="26" t="str">
-        <x:v>Đồng bộ sang giỏ: Thêm lặp combo</x:v>
+        <x:v>Kiểm tra nút MUA NGAY ở kích thước điện thoại</x:v>
       </x:c>
       <x:c r="E94" s="30" t="str">
-        <x:v>Consistency</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F94" s="30" t="str">
-        <x:v>State / UI Consistency</x:v>
+        <x:v>Boundary Value</x:v>
       </x:c>
       <x:c r="G94" s="30" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H94" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Dùng viewport 390 x 844, không tạo đơn thật; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I94" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Chuyển sản phẩm/gói đã chọn vào giỏ (không đặt hàng); tình huống: Thêm lặp combo.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Dùng viewport 390 x 844, không tạo đơn thật.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Mở trang S25 Ultra 256GB, chọn màu khả dụng và nhấn MUA NGAY.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J94" s="26" t="str">
-        <x:v>Thêm lặp combo  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>Mobile 390×844; Bạc</x:v>
       </x:c>
       <x:c r="K94" s="26" t="str">
-        <x:v>Giỏ phản ánh đúng món mua kèm, giá, số lượng và ưu đãi.</x:v>
+        <x:v>Giao diện mua trên mobile truy cập được, CTA không tràn; luồng chuyển đến vẫn đúng SKU; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L94" s="26"/>
       <x:c r="M94" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N94" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O94" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P94" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q94" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="69" customHeight="1">
@@ -13392,50 +13501,51 @@
         <x:v>D06</x:v>
       </x:c>
       <x:c r="C95" s="26" t="str">
-        <x:v>Sản phẩm mua kèm và ưu đãi mua kèm</x:v>
+        <x:v>Mua ngay và kiểm tra thông tin sản phẩm trước đặt hàng</x:v>
       </x:c>
       <x:c r="D95" s="26" t="str">
-        <x:v>Đồng bộ sang giỏ: Xóa máy chính khỏi giỏ</x:v>
+        <x:v>Dừng ở bước trước xác nhận đơn hàng</x:v>
       </x:c>
       <x:c r="E95" s="30" t="str">
-        <x:v>Consistency</x:v>
+        <x:v>Positive</x:v>
       </x:c>
       <x:c r="F95" s="30" t="str">
-        <x:v>State / UI Consistency</x:v>
+        <x:v>Decision Table</x:v>
       </x:c>
       <x:c r="G95" s="30" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H95" s="26" t="str">
-        <x:v>Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.</x:v>
+        <x:v>Trang Samsung S25 Ultra có nút MUA NGAY; Mở luồng MUA NGAY cho 256GB, chưa điền thông tin người nhận; không đặt hàng.</x:v>
       </x:c>
       <x:c r="I95" s="26" t="str">
-        <x:v>1. Mở https://didongviet.vn/.
-2. Chuẩn bị: Mẫu sản phẩm có mục mua kèm/ưu đãi mua kèm; chưa xác nhận tính năng cho mọi SKU.
-3. Chuyển sản phẩm/gói đã chọn vào giỏ (không đặt hàng); tình huống: Xóa máy chính khỏi giỏ.
-4. Quan sát phản hồi và đối chiếu expected result, KHÔNG thực hiện giao dịch thật.</x:v>
+        <x:v>1. Mở https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html.
+2. Mở luồng MUA NGAY cho 256GB, chưa điền thông tin người nhận.
+3. Ghi nhận phiên bản/màu/giá ở trang chi tiết.
+4. Quan sát khu vực thông tin/tóm tắt đơn khi tới bước mua; dừng mà không nhấn nút đặt hàng.
+5. Đối chiếu kết quả; KHÔNG đặt hàng hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="J95" s="26" t="str">
-        <x:v>Xóa máy chính khỏi giỏ  |  Giá trị thực: ghi lại sau khi kiểm tra website</x:v>
+        <x:v>256GB; Titan Xanh; không nhập PII/không submit</x:v>
       </x:c>
       <x:c r="K95" s="26" t="str">
-        <x:v>Giỏ phản ánh đúng món mua kèm, giá, số lượng và ưu đãi.</x:v>
+        <x:v>Không có màn hình báo tạo đơn hoặc giao dịch thành công do chỉ nhấn MUA NGAY; dừng trước submit; không tự tạo đơn hoặc thanh toán.</x:v>
       </x:c>
       <x:c r="L95" s="26"/>
       <x:c r="M95" s="30" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N95" s="30" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="O95" s="30" t="str">
-        <x:v>Cần xác minh</x:v>
+        <x:v>Đã thấy bộ lọc</x:v>
       </x:c>
       <x:c r="P95" s="26" t="str">
-        <x:v>Chỉ thực hiện case khi giao diện thật có lựa chọn tương ứng. | CHỈ THỰC HIỆN nếu UI và dữ liệu kịch bản thật sự có.</x:v>
+        <x:v>Thay F06 cũ; xác nhận trên giao diện có Tất cả, Có hình ảnh, các mức 1–5 sao và Sắp xếp theo. Không submit.</x:v>
       </x:c>
       <x:c r="Q95" s="26" t="str">
-        <x:v>https://didongviet.vn/</x:v>
+        <x:v>https://didongviet.vn/dien-thoai/samsung-galaxy-s25-ultra-5g-256gb.html</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28867,7 +28977,7 @@
     </x:row>
     <x:row r="2" ht="31" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>Bộ 450 test case dự thảo • 15 chức năng • 5 thành viên • Không chứa kết quả test đã chạy</x:v>
+        <x:v>450 test case / 15 chức năng • F06 mới: MUA NGAY, giữ SKU/giá trước đặt hàng, thuộc nhóm F04/F05 • F04 TV2 PASS 30/30</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
         <x:v>Bộ 450 test case dự thảo • 15 chức năng • 5 thành viên • Không chứa kết quả test đã chạy</x:v>
@@ -28960,13 +29070,13 @@
       </x:c>
       <x:c r="B8" s="26" t="n">
         <x:f>SUM('PHAN CONG'!I6:I20)</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
         <x:v>Chỉ tăng sau khi chạy thực tế</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Theo kết quả F04 TV2 xác nhận</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -28975,13 +29085,13 @@
       </x:c>
       <x:c r="B9" s="26" t="n">
         <x:f>SUM('PHAN CONG'!J6:J20)</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="26" t="str">
         <x:v>Không giả kết quả</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>30 Passed – F04 TV2</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -28990,10 +29100,10 @@
       </x:c>
       <x:c r="B10" s="26" t="n">
         <x:f>450-('TV1 - TEST CASE'!J3+'TV2 - TEST CASE'!J3+'TV3 - TEST CASE'!J3+'TV4 - TEST CASE'!J3+'TV5 - TEST CASE'!J3)</x:f>
-        <x:v>450</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="C10" s="26" t="str">
-        <x:v>Kiểm tra UI trước khi dùng chính thức</x:v>
+        <x:v>Rà soát UI chưa chạy; đã thấy nút MUA NGAY tại trang Samsung, cần xác minh luồng sau nhấn</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>Cần rà soát</x:v>
@@ -29092,11 +29202,11 @@
       </x:c>
       <x:c r="E17" s="26" t="n">
         <x:f>'TV2 - TEST CASE'!D3</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F17" s="26" t="n">
         <x:f>'TV2 - TEST CASE'!F3</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
         <x:v>F04 - Lựa chọn phiên bản, dung lượng và màu sắc</x:v>
@@ -29196,11 +29306,11 @@
       </x:c>
       <x:c r="E22" s="32" t="n">
         <x:f>SUM(E16:E20)</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F22" s="32" t="n">
         <x:f>SUM(F16:F20)</x:f>
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G22" s="32" t="str">
         <x:v>5 x 30 TC tuần đầu</x:v>

</xml_diff>